<commit_message>
Week 5: turnover and two-predictor sheets, Brady brief, deadline data, worksheets refresh on /update
</commit_message>
<xml_diff>
--- a/weeks/week05/data/hand-build-regression-worksheet.xlsx
+++ b/weeks/week05/data/hand-build-regression-worksheet.xlsx
@@ -68,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -78,14 +78,8 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1208,25 +1202,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The same ten team-games. Slope and intercept are given here so this sheet stands on its own; they match what the first sheet produces.</t>
+          <t>The same ten team-games, plus each team's turnover differential that game: takeaways minus giveaways, from nflverse play-by-play.</t>
         </is>
       </c>
     </row>
@@ -1243,35 +1238,40 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>Turnover differential (second x)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>Margin (y)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Predicted margin</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Residual squared</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -1287,14 +1287,17 @@
         <v>46</v>
       </c>
       <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
         <v>6</v>
       </c>
-      <c r="D3" s="4" t="n"/>
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
-      <c r="H3" s="5" t="n"/>
+      <c r="G3" s="4" t="n"/>
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="5" t="n"/>
+      <c r="K3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1306,14 +1309,17 @@
         <v>24</v>
       </c>
       <c r="C4" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D4" t="n">
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="n"/>
-      <c r="H4" s="5" t="n"/>
+      <c r="G4" s="4" t="n"/>
       <c r="I4" s="5" t="n"/>
       <c r="J4" s="5" t="n"/>
+      <c r="K4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1327,12 +1333,15 @@
       <c r="C5" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="4" t="n"/>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="G5" s="4" t="n"/>
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1344,14 +1353,17 @@
         <v>31</v>
       </c>
       <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
         <v>16</v>
       </c>
-      <c r="D6" s="4" t="n"/>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="4" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="G6" s="4" t="n"/>
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1363,14 +1375,17 @@
         <v>19</v>
       </c>
       <c r="C7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D7" t="n">
         <v>-3</v>
       </c>
-      <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="G7" s="4" t="n"/>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1382,14 +1397,17 @@
         <v>23</v>
       </c>
       <c r="C8" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D8" t="n">
         <v>-15</v>
       </c>
-      <c r="D8" s="4" t="n"/>
       <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="G8" s="4" t="n"/>
       <c r="I8" s="5" t="n"/>
       <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1401,14 +1419,17 @@
         <v>19</v>
       </c>
       <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
         <v>-3</v>
       </c>
-      <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="G9" s="4" t="n"/>
       <c r="I9" s="5" t="n"/>
       <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1420,14 +1441,17 @@
         <v>24</v>
       </c>
       <c r="C10" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D10" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="4" t="n"/>
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="G10" s="4" t="n"/>
       <c r="I10" s="5" t="n"/>
       <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1439,14 +1463,17 @@
         <v>45</v>
       </c>
       <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
         <v>38</v>
       </c>
-      <c r="D11" s="4" t="n"/>
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="G11" s="4" t="n"/>
       <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1458,345 +1485,466 @@
         <v>25</v>
       </c>
       <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
         <v>24</v>
       </c>
-      <c r="D12" s="4" t="n"/>
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
-      <c r="H12" s="5" t="n"/>
+      <c r="G12" s="4" t="n"/>
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="E14" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Your answer</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Slope, SLOPE(y range, x range)</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="5" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Intercept, INTERCEPT(y range, x range)</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="5" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Sum of squared residuals</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="5" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Residual standard error: SQRT of that sum divided by (n minus 2), n = 10</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="5" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Check it with Excel, STEYX(y range, x range)</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="5" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Standard error of the slope: residual standard error divided by SQRT of the sum of squared x deviations</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="5" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>t: slope divided by its standard error</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="5" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="5" t="n"/>
     </row>
     <row r="22">
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>p-value, two-sided: T.DIST.2T(ABS(t), n minus 2)</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="5" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="5" t="n"/>
     </row>
     <row r="23">
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Lower end of the 95%% interval: slope minus T.INV.2T(0.05, n minus 2) times the standard error</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="5" t="n"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Lower end of the 95% interval: slope minus T.INV.2T(0.05, n minus 2) times the standard error</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Upper end of the 95%% interval</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="5" t="n"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Upper end of the 95% interval</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="5" t="n"/>
     </row>
     <row r="25">
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Standard error of the slope from Excel, INDEX(LINEST(y range, x range, TRUE, TRUE), 2, 1)</t>
         </is>
       </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="5" t="n"/>
-    </row>
-    <row r="26" ht="60" customHeight="1">
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Would you tell a coach these ten games show that rushing more moves the margin? One sentence, and say which number above you leaned on.</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Turnover differential as x instead: its slope, SLOPE(y range, turnover range)</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Its standard error, INDEX(LINEST(y range, turnover range, TRUE, TRUE), 2, 1)</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="5" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>Every number here is one Excel prints when you run Data Analysis, Regression, or LINEST. Build each one yourself, then confirm the standard error against LINEST.</t>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Its p-value, two-sided: T.DIST.2T(ABS(slope divided by standard error), n minus 2)</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Lower end of its 95% interval</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Upper end of its 95% interval</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Standard deviation of rush attempts across the ten games, STDEV.S</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Standard deviation of turnover differential, STDEV.S</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Margin moved by one standard deviation of rush attempts: the rush slope times that standard deviation</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Margin moved by one standard deviation of turnover differential</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Every number in the first block is one Excel prints when you run Data Analysis, Regression, or LINEST. Build each one yourself, then confirm the standard error against LINEST.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H3">
+  <conditionalFormatting sqref="I3">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(ISNUMBER(D3),ABS(D3-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B3)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B3)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I3">
+      <formula>AND(ISNUMBER(E3),ABS(E3-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B3)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B3)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3">
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>AND(ISNUMBER(E3),ABS(E3-((C3-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B3))))&lt;=MAX(0.02*ABS((C3-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B3))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J3">
+      <formula>AND(ISNUMBER(F3),ABS(F3-((D3-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B3))))&lt;=MAX(0.02*ABS((D3-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B3))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>AND(ISNUMBER(F3),ABS(F3-(((C3-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B3))^2)))&lt;=MAX(0.02*ABS(((C3-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B3))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H4">
+      <formula>AND(ISNUMBER(G3),ABS(G3-(((D3-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B3))^2)))&lt;=MAX(0.02*ABS(((D3-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B3))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4">
     <cfRule type="expression" priority="4" dxfId="0">
-      <formula>AND(ISNUMBER(D4),ABS(D4-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B4)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B4)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I4">
+      <formula>AND(ISNUMBER(E4),ABS(E4-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B4)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B4)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J4">
     <cfRule type="expression" priority="5" dxfId="0">
-      <formula>AND(ISNUMBER(E4),ABS(E4-((C4-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B4))))&lt;=MAX(0.02*ABS((C4-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B4))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J4">
+      <formula>AND(ISNUMBER(F4),ABS(F4-((D4-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B4))))&lt;=MAX(0.02*ABS((D4-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B4))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
     <cfRule type="expression" priority="6" dxfId="0">
-      <formula>AND(ISNUMBER(F4),ABS(F4-(((C4-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B4))^2)))&lt;=MAX(0.02*ABS(((C4-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B4))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H5">
+      <formula>AND(ISNUMBER(G4),ABS(G4-(((D4-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B4))^2)))&lt;=MAX(0.02*ABS(((D4-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B4))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5">
     <cfRule type="expression" priority="7" dxfId="0">
-      <formula>AND(ISNUMBER(D5),ABS(D5-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B5)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B5)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I5">
+      <formula>AND(ISNUMBER(E5),ABS(E5-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B5)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B5)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5">
     <cfRule type="expression" priority="8" dxfId="0">
-      <formula>AND(ISNUMBER(E5),ABS(E5-((C5-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B5))))&lt;=MAX(0.02*ABS((C5-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B5))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5">
+      <formula>AND(ISNUMBER(F5),ABS(F5-((D5-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B5))))&lt;=MAX(0.02*ABS((D5-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B5))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5">
     <cfRule type="expression" priority="9" dxfId="0">
-      <formula>AND(ISNUMBER(F5),ABS(F5-(((C5-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B5))^2)))&lt;=MAX(0.02*ABS(((C5-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B5))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H6">
+      <formula>AND(ISNUMBER(G5),ABS(G5-(((D5-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B5))^2)))&lt;=MAX(0.02*ABS(((D5-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B5))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6">
     <cfRule type="expression" priority="10" dxfId="0">
-      <formula>AND(ISNUMBER(D6),ABS(D6-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B6)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B6)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I6">
+      <formula>AND(ISNUMBER(E6),ABS(E6-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B6)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B6)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J6">
     <cfRule type="expression" priority="11" dxfId="0">
-      <formula>AND(ISNUMBER(E6),ABS(E6-((C6-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B6))))&lt;=MAX(0.02*ABS((C6-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B6))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J6">
+      <formula>AND(ISNUMBER(F6),ABS(F6-((D6-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B6))))&lt;=MAX(0.02*ABS((D6-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B6))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6">
     <cfRule type="expression" priority="12" dxfId="0">
-      <formula>AND(ISNUMBER(F6),ABS(F6-(((C6-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B6))^2)))&lt;=MAX(0.02*ABS(((C6-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B6))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H7">
+      <formula>AND(ISNUMBER(G6),ABS(G6-(((D6-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B6))^2)))&lt;=MAX(0.02*ABS(((D6-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B6))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I7">
     <cfRule type="expression" priority="13" dxfId="0">
-      <formula>AND(ISNUMBER(D7),ABS(D7-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B7)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B7)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I7">
+      <formula>AND(ISNUMBER(E7),ABS(E7-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B7)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B7)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7">
     <cfRule type="expression" priority="14" dxfId="0">
-      <formula>AND(ISNUMBER(E7),ABS(E7-((C7-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B7))))&lt;=MAX(0.02*ABS((C7-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B7))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J7">
+      <formula>AND(ISNUMBER(F7),ABS(F7-((D7-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B7))))&lt;=MAX(0.02*ABS((D7-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B7))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K7">
     <cfRule type="expression" priority="15" dxfId="0">
-      <formula>AND(ISNUMBER(F7),ABS(F7-(((C7-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B7))^2)))&lt;=MAX(0.02*ABS(((C7-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B7))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H8">
+      <formula>AND(ISNUMBER(G7),ABS(G7-(((D7-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B7))^2)))&lt;=MAX(0.02*ABS(((D7-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B7))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I8">
     <cfRule type="expression" priority="16" dxfId="0">
-      <formula>AND(ISNUMBER(D8),ABS(D8-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B8)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B8)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I8">
+      <formula>AND(ISNUMBER(E8),ABS(E8-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B8)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B8)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J8">
     <cfRule type="expression" priority="17" dxfId="0">
-      <formula>AND(ISNUMBER(E8),ABS(E8-((C8-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B8))))&lt;=MAX(0.02*ABS((C8-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B8))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J8">
+      <formula>AND(ISNUMBER(F8),ABS(F8-((D8-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B8))))&lt;=MAX(0.02*ABS((D8-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B8))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K8">
     <cfRule type="expression" priority="18" dxfId="0">
-      <formula>AND(ISNUMBER(F8),ABS(F8-(((C8-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B8))^2)))&lt;=MAX(0.02*ABS(((C8-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B8))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H9">
+      <formula>AND(ISNUMBER(G8),ABS(G8-(((D8-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B8))^2)))&lt;=MAX(0.02*ABS(((D8-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B8))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I9">
     <cfRule type="expression" priority="19" dxfId="0">
-      <formula>AND(ISNUMBER(D9),ABS(D9-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B9)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B9)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I9">
+      <formula>AND(ISNUMBER(E9),ABS(E9-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B9)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B9)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J9">
     <cfRule type="expression" priority="20" dxfId="0">
-      <formula>AND(ISNUMBER(E9),ABS(E9-((C9-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B9))))&lt;=MAX(0.02*ABS((C9-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B9))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J9">
+      <formula>AND(ISNUMBER(F9),ABS(F9-((D9-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B9))))&lt;=MAX(0.02*ABS((D9-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B9))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9">
     <cfRule type="expression" priority="21" dxfId="0">
-      <formula>AND(ISNUMBER(F9),ABS(F9-(((C9-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B9))^2)))&lt;=MAX(0.02*ABS(((C9-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B9))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H10">
+      <formula>AND(ISNUMBER(G9),ABS(G9-(((D9-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B9))^2)))&lt;=MAX(0.02*ABS(((D9-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B9))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I10">
     <cfRule type="expression" priority="22" dxfId="0">
-      <formula>AND(ISNUMBER(D10),ABS(D10-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B10)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B10)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I10">
+      <formula>AND(ISNUMBER(E10),ABS(E10-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B10)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B10)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J10">
     <cfRule type="expression" priority="23" dxfId="0">
-      <formula>AND(ISNUMBER(E10),ABS(E10-((C10-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B10))))&lt;=MAX(0.02*ABS((C10-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B10))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J10">
+      <formula>AND(ISNUMBER(F10),ABS(F10-((D10-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B10))))&lt;=MAX(0.02*ABS((D10-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B10))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K10">
     <cfRule type="expression" priority="24" dxfId="0">
-      <formula>AND(ISNUMBER(F10),ABS(F10-(((C10-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B10))^2)))&lt;=MAX(0.02*ABS(((C10-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B10))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H11">
+      <formula>AND(ISNUMBER(G10),ABS(G10-(((D10-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B10))^2)))&lt;=MAX(0.02*ABS(((D10-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B10))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I11">
     <cfRule type="expression" priority="25" dxfId="0">
-      <formula>AND(ISNUMBER(D11),ABS(D11-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B11)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B11)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I11">
+      <formula>AND(ISNUMBER(E11),ABS(E11-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B11)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B11)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J11">
     <cfRule type="expression" priority="26" dxfId="0">
-      <formula>AND(ISNUMBER(E11),ABS(E11-((C11-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B11))))&lt;=MAX(0.02*ABS((C11-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B11))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11">
+      <formula>AND(ISNUMBER(F11),ABS(F11-((D11-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B11))))&lt;=MAX(0.02*ABS((D11-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B11))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
     <cfRule type="expression" priority="27" dxfId="0">
-      <formula>AND(ISNUMBER(F11),ABS(F11-(((C11-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B11))^2)))&lt;=MAX(0.02*ABS(((C11-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B11))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H12">
+      <formula>AND(ISNUMBER(G11),ABS(G11-(((D11-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B11))^2)))&lt;=MAX(0.02*ABS(((D11-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B11))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I12">
     <cfRule type="expression" priority="28" dxfId="0">
-      <formula>AND(ISNUMBER(D12),ABS(D12-((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B12)))&lt;=MAX(0.02*ABS((INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B12)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I12">
+      <formula>AND(ISNUMBER(E12),ABS(E12-((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B12)))&lt;=MAX(0.02*ABS((INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B12)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J12">
     <cfRule type="expression" priority="29" dxfId="0">
-      <formula>AND(ISNUMBER(E12),ABS(E12-((C12-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B12))))&lt;=MAX(0.02*ABS((C12-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B12))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J12">
+      <formula>AND(ISNUMBER(F12),ABS(F12-((D12-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B12))))&lt;=MAX(0.02*ABS((D12-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B12))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
     <cfRule type="expression" priority="30" dxfId="0">
-      <formula>AND(ISNUMBER(F12),ABS(F12-(((C12-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B12))^2)))&lt;=MAX(0.02*ABS(((C12-(INTERCEPT($C$3:$C$12,$B$3:$B$12)+SLOPE($C$3:$C$12,$B$3:$B$12)*B12))^2)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F15">
+      <formula>AND(ISNUMBER(G12),ABS(G12-(((D12-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B12))^2)))&lt;=MAX(0.02*ABS(((D12-(INTERCEPT($D$3:$D$12,$B$3:$B$12)+SLOPE($D$3:$D$12,$B$3:$B$12)*B12))^2)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G15">
     <cfRule type="expression" priority="31" dxfId="0">
-      <formula>AND(ISNUMBER(E15),ABS(E15-(SLOPE($C$3:$C$12,$B$3:$B$12)))&lt;=MAX(0.02*ABS(SLOPE($C$3:$C$12,$B$3:$B$12)),0.005))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F16">
+      <formula>AND(ISNUMBER(F15),ABS(F15-(SLOPE($D$3:$D$12,$B$3:$B$12)))&lt;=MAX(0.02*ABS(SLOPE($D$3:$D$12,$B$3:$B$12)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16">
     <cfRule type="expression" priority="32" dxfId="0">
-      <formula>AND(ISNUMBER(E16),ABS(E16-(INTERCEPT($C$3:$C$12,$B$3:$B$12)))&lt;=MAX(0.02*ABS(INTERCEPT($C$3:$C$12,$B$3:$B$12)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F17">
+      <formula>AND(ISNUMBER(F16),ABS(F16-(INTERCEPT($D$3:$D$12,$B$3:$B$12)))&lt;=MAX(0.02*ABS(INTERCEPT($D$3:$D$12,$B$3:$B$12)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17">
     <cfRule type="expression" priority="33" dxfId="0">
-      <formula>AND(ISNUMBER(E17),ABS(E17-((DEVSQ($C$3:$C$12)-SLOPE($C$3:$C$12,$B$3:$B$12)^2*DEVSQ($B$3:$B$12))))&lt;=MAX(0.02*ABS((DEVSQ($C$3:$C$12)-SLOPE($C$3:$C$12,$B$3:$B$12)^2*DEVSQ($B$3:$B$12))),1.0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F18">
+      <formula>AND(ISNUMBER(F17),ABS(F17-((DEVSQ($D$3:$D$12)-SLOPE($D$3:$D$12,$B$3:$B$12)^2*DEVSQ($B$3:$B$12))))&lt;=MAX(0.02*ABS((DEVSQ($D$3:$D$12)-SLOPE($D$3:$D$12,$B$3:$B$12)^2*DEVSQ($B$3:$B$12))),1.0))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18">
     <cfRule type="expression" priority="34" dxfId="0">
-      <formula>AND(ISNUMBER(E18),ABS(E18-(STEYX($C$3:$C$12,$B$3:$B$12)))&lt;=MAX(0.02*ABS(STEYX($C$3:$C$12,$B$3:$B$12)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F19">
+      <formula>AND(ISNUMBER(F18),ABS(F18-(STEYX($D$3:$D$12,$B$3:$B$12)))&lt;=MAX(0.02*ABS(STEYX($D$3:$D$12,$B$3:$B$12)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19">
     <cfRule type="expression" priority="35" dxfId="0">
-      <formula>AND(ISNUMBER(E19),ABS(E19-(STEYX($C$3:$C$12,$B$3:$B$12)))&lt;=MAX(0.02*ABS(STEYX($C$3:$C$12,$B$3:$B$12)),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F20">
+      <formula>AND(ISNUMBER(F19),ABS(F19-(STEYX($D$3:$D$12,$B$3:$B$12)))&lt;=MAX(0.02*ABS(STEYX($D$3:$D$12,$B$3:$B$12)),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G20">
     <cfRule type="expression" priority="36" dxfId="0">
-      <formula>AND(ISNUMBER(E20),ABS(E20-((STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))))&lt;=MAX(0.02*ABS((STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))),0.005))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F21">
+      <formula>AND(ISNUMBER(F20),ABS(F20-((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))))&lt;=MAX(0.02*ABS((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G21">
     <cfRule type="expression" priority="37" dxfId="0">
-      <formula>AND(ISNUMBER(E21),ABS(E21-((SLOPE($C$3:$C$12,$B$3:$B$12)/(STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($C$3:$C$12,$B$3:$B$12)/(STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F22">
+      <formula>AND(ISNUMBER(F21),ABS(F21-((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G22">
     <cfRule type="expression" priority="38" dxfId="0">
-      <formula>AND(ISNUMBER(E22),ABS(E22-(_xlfn.T.DIST.2T(ABS((SLOPE($C$3:$C$12,$B$3:$B$12)/(STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),8)))&lt;=MAX(0.02*ABS(_xlfn.T.DIST.2T(ABS((SLOPE($C$3:$C$12,$B$3:$B$12)/(STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),8)),0.005))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F23">
+      <formula>AND(ISNUMBER(F22),ABS(F22-(_xlfn.T.DIST.2T(ABS((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),8)))&lt;=MAX(0.02*ABS(_xlfn.T.DIST.2T(ABS((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),8)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23">
     <cfRule type="expression" priority="39" dxfId="0">
-      <formula>AND(ISNUMBER(E23),ABS(E23-((SLOPE($C$3:$C$12,$B$3:$B$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($C$3:$C$12,$B$3:$B$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F24">
+      <formula>AND(ISNUMBER(F23),ABS(F23-((SLOPE($D$3:$D$12,$B$3:$B$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G24">
     <cfRule type="expression" priority="40" dxfId="0">
-      <formula>AND(ISNUMBER(E24),ABS(E24-((SLOPE($C$3:$C$12,$B$3:$B$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($C$3:$C$12,$B$3:$B$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F25">
+      <formula>AND(ISNUMBER(F24),ABS(F24-((SLOPE($D$3:$D$12,$B$3:$B$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G25">
     <cfRule type="expression" priority="41" dxfId="0">
-      <formula>AND(ISNUMBER(E25),ABS(E25-((STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))))&lt;=MAX(0.02*ABS((STEYX($C$3:$C$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))),0.005))</formula>
+      <formula>AND(ISNUMBER(F25),ABS(F25-((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))))&lt;=MAX(0.02*ABS((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G26">
+    <cfRule type="expression" priority="42" dxfId="0">
+      <formula>AND(ISNUMBER(F26),ABS(F26-(SLOPE($D$3:$D$12,$C$3:$C$12)))&lt;=MAX(0.02*ABS(SLOPE($D$3:$D$12,$C$3:$C$12)),0.01))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G27">
+    <cfRule type="expression" priority="43" dxfId="0">
+      <formula>AND(ISNUMBER(F27),ABS(F27-((STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))))&lt;=MAX(0.02*ABS((STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))),0.01))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G28">
+    <cfRule type="expression" priority="44" dxfId="0">
+      <formula>AND(ISNUMBER(F28),ABS(F28-(_xlfn.T.DIST.2T(ABS(SLOPE($D$3:$D$12,$C$3:$C$12)/(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))),8)))&lt;=MAX(0.02*ABS(_xlfn.T.DIST.2T(ABS(SLOPE($D$3:$D$12,$C$3:$C$12)/(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))),8)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G29">
+    <cfRule type="expression" priority="45" dxfId="0">
+      <formula>AND(ISNUMBER(F29),ABS(F29-((SLOPE($D$3:$D$12,$C$3:$C$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$C$3:$C$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12))))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30">
+    <cfRule type="expression" priority="46" dxfId="0">
+      <formula>AND(ISNUMBER(F30),ABS(F30-((SLOPE($D$3:$D$12,$C$3:$C$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$C$3:$C$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12))))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G31">
+    <cfRule type="expression" priority="47" dxfId="0">
+      <formula>AND(ISNUMBER(F31),ABS(F31-(_xlfn.STDEV.S($B$3:$B$12)))&lt;=MAX(0.02*ABS(_xlfn.STDEV.S($B$3:$B$12)),0.01))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G32">
+    <cfRule type="expression" priority="48" dxfId="0">
+      <formula>AND(ISNUMBER(F32),ABS(F32-(_xlfn.STDEV.S($C$3:$C$12)))&lt;=MAX(0.02*ABS(_xlfn.STDEV.S($C$3:$C$12)),0.01))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G33">
+    <cfRule type="expression" priority="49" dxfId="0">
+      <formula>AND(ISNUMBER(F33),ABS(F33-((SLOPE($D$3:$D$12,$B$3:$B$12)*_xlfn.STDEV.S($B$3:$B$12))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)*_xlfn.STDEV.S($B$3:$B$12))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G34">
+    <cfRule type="expression" priority="50" dxfId="0">
+      <formula>AND(ISNUMBER(F34),ABS(F34-((SLOPE($D$3:$D$12,$C$3:$C$12)*_xlfn.STDEV.S($C$3:$C$12))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$C$3:$C$12)*_xlfn.STDEV.S($C$3:$C$12))),0.05))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1867,21 +2015,21 @@
           <t>Arizona Diamondbacks</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="7" t="n">
         <v>0.337</v>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="7" t="n">
         <v>0.44</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="7" t="n">
         <v>5.469</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Coefficient on OBP: INDEX(LINEST(y range, both x columns, TRUE, TRUE), 1, 2). LINEST lists the x coefficients in reverse column order.</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="n"/>
+          <t>How closely OBP and SLG move together across the 30 teams, CORREL(OBP range, SLG range)</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -1890,21 +2038,21 @@
           <t>Atlanta Braves</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="7" t="n">
         <v>0.309</v>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="7" t="n">
         <v>0.415</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="7" t="n">
         <v>4.346</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Coefficient on SLG: INDEX(LINEST(...), 1, 1)</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="n"/>
+          <t>OBP alone: its slope, SLOPE(y range, OBP range)</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="n"/>
       <c r="H4" s="5" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
@@ -1913,21 +2061,21 @@
           <t>Baltimore Orioles</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="7" t="n">
         <v>0.315</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="7" t="n">
         <v>0.435</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="7" t="n">
         <v>4.852</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Intercept: INDEX(LINEST(...), 1, 3)</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="n"/>
+          <t>OBP alone: R squared, RSQ(y range, OBP range)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
     <row r="6" ht="32" customHeight="1">
@@ -1936,21 +2084,21 @@
           <t>Boston Red Sox</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="7" t="n">
         <v>0.319</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="7" t="n">
         <v>0.423</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="7" t="n">
         <v>4.636</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Standard error of the OBP coefficient: INDEX(LINEST(...), 2, 2)</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="n"/>
+          <t>SLG alone: its slope, SLOPE(y range, SLG range)</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="n"/>
       <c r="H6" s="5" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -1959,21 +2107,21 @@
           <t>Chicago Cubs</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="7" t="n">
         <v>0.317</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="7" t="n">
         <v>0.393</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="7" t="n">
         <v>4.543</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Standard error of the SLG coefficient: INDEX(LINEST(...), 2, 1)</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="n"/>
+          <t>SLG alone: R squared, RSQ(y range, SLG range)</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="n"/>
       <c r="H7" s="5" t="n"/>
     </row>
     <row r="8" ht="32" customHeight="1">
@@ -1982,21 +2130,21 @@
           <t>Chicago White Sox</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="7" t="n">
         <v>0.278</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="7" t="n">
         <v>0.34</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="7" t="n">
         <v>3.13</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>t for OBP: coefficient divided by its standard error</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="n"/>
+          <t>Both together. Coefficient on OBP: INDEX(LINEST(y range, both x columns, TRUE, TRUE), 1, 2). LINEST lists the x coefficients in reverse column order.</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="n"/>
       <c r="H8" s="5" t="n"/>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -2005,21 +2153,21 @@
           <t>Cincinnati Reds</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="7" t="n">
         <v>0.305</v>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="7" t="n">
         <v>0.388</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="7" t="n">
         <v>4.315</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>t for SLG</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="n"/>
+          <t>Coefficient on SLG: INDEX(LINEST(...), 1, 1)</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="n"/>
       <c r="H9" s="5" t="n"/>
     </row>
     <row r="10" ht="32" customHeight="1">
@@ -2028,21 +2176,21 @@
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="7" t="n">
         <v>0.307</v>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="7" t="n">
         <v>0.395</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="7" t="n">
         <v>4.398</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>p-value for OBP: T.DIST.2T(ABS(t), n minus 3), n = 30</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="n"/>
+          <t>Intercept: INDEX(LINEST(...), 1, 3)</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="n"/>
       <c r="H10" s="5" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
@@ -2051,21 +2199,21 @@
           <t>Colorado Rockies</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="7" t="n">
         <v>0.304</v>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="7" t="n">
         <v>4.21</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>p-value for SLG</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="n"/>
+          <t>Standard error of the OBP coefficient: INDEX(LINEST(...), 2, 2)</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="n"/>
       <c r="H11" s="5" t="n"/>
     </row>
     <row r="12" ht="32" customHeight="1">
@@ -2074,21 +2222,21 @@
           <t>Detroit Tigers</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="7" t="n">
         <v>0.385</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="7" t="n">
         <v>4.21</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>R squared: INDEX(LINEST(...), 3, 1)</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="n"/>
+          <t>Standard error of the SLG coefficient: INDEX(LINEST(...), 2, 1)</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="n"/>
       <c r="H12" s="5" t="n"/>
     </row>
     <row r="13" ht="32" customHeight="1">
@@ -2097,21 +2245,21 @@
           <t>Houston Astros</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="7" t="n">
         <v>0.322</v>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="7" t="n">
         <v>0.418</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="7" t="n">
         <v>4.596</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Standard deviation of OBP across the 30 teams, STDEV.S</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="n"/>
+          <t>t for OBP: coefficient divided by its standard error</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="n"/>
       <c r="H13" s="5" t="n"/>
     </row>
     <row r="14" ht="32" customHeight="1">
@@ -2120,21 +2268,21 @@
           <t>Kansas City Royals</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="7" t="n">
         <v>0.306</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="7" t="n">
         <v>0.403</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="7" t="n">
         <v>4.537</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Standard deviation of SLG, STDEV.S</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="n"/>
+          <t>t for SLG</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="n"/>
       <c r="H14" s="5" t="n"/>
     </row>
     <row r="15" ht="32" customHeight="1">
@@ -2143,21 +2291,21 @@
           <t>Los Angeles Angels</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="7" t="n">
         <v>0.301</v>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="7" t="n">
         <v>0.369</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="7" t="n">
         <v>3.92</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Runs per game from one standard deviation of OBP: coefficient times that standard deviation</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="n"/>
+          <t>p-value for OBP: T.DIST.2T(ABS(t), n minus 3), n = 30</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="n"/>
       <c r="H15" s="5" t="n"/>
     </row>
     <row r="16" ht="32" customHeight="1">
@@ -2166,44 +2314,45 @@
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="7" t="n">
         <v>0.335</v>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="7" t="n">
         <v>0.446</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="7" t="n">
         <v>5.198</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Runs per game from one standard deviation of SLG</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="n"/>
+          <t>p-value for SLG</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="n"/>
       <c r="H16" s="5" t="n"/>
     </row>
-    <row r="17" ht="75" customHeight="1">
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>Miami Marlins</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="7" t="n">
         <v>0.378</v>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D17" s="7" t="n">
         <v>3.932</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>The OBP coefficient is about twice the SLG coefficient. Which of the two matters more to a team's runs, and what is the case for each answer? Two sentences.</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="n"/>
+          <t>R squared with both: INDEX(LINEST(...), 3, 1)</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2211,13 +2360,13 @@
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="7" t="n">
         <v>0.326</v>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="7" t="n">
         <v>0.403</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="7" t="n">
         <v>4.796</v>
       </c>
     </row>
@@ -2227,13 +2376,13 @@
           <t>Minnesota Twins</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="7" t="n">
         <v>0.315</v>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="7" t="n">
         <v>0.411</v>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="D19" s="7" t="n">
         <v>4.58</v>
       </c>
     </row>
@@ -2243,13 +2392,13 @@
           <t>New York Mets</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="7" t="n">
         <v>0.319</v>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="7" t="n">
         <v>0.415</v>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D20" s="7" t="n">
         <v>4.741</v>
       </c>
     </row>
@@ -2259,13 +2408,13 @@
           <t>New York Yankees</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n">
+      <c r="B21" s="7" t="n">
         <v>0.333</v>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="7" t="n">
         <v>0.429</v>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D21" s="7" t="n">
         <v>5.031</v>
       </c>
     </row>
@@ -2275,13 +2424,13 @@
           <t>Oakland Athletics</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="7" t="n">
         <v>0.301</v>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C22" s="7" t="n">
         <v>0.393</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D22" s="7" t="n">
         <v>3.969</v>
       </c>
     </row>
@@ -2291,13 +2440,13 @@
           <t>Philadelphia Phillies</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B23" s="7" t="n">
         <v>0.325</v>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C23" s="7" t="n">
         <v>0.425</v>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D23" s="7" t="n">
         <v>4.84</v>
       </c>
     </row>
@@ -2307,13 +2456,13 @@
           <t>Pittsburgh Pirates</t>
         </is>
       </c>
-      <c r="B24" s="8" t="n">
+      <c r="B24" s="7" t="n">
         <v>0.301</v>
       </c>
-      <c r="C24" s="8" t="n">
+      <c r="C24" s="7" t="n">
         <v>0.371</v>
       </c>
-      <c r="D24" s="8" t="n">
+      <c r="D24" s="7" t="n">
         <v>4.105</v>
       </c>
     </row>
@@ -2323,13 +2472,13 @@
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="B25" s="8" t="n">
+      <c r="B25" s="7" t="n">
         <v>0.324</v>
       </c>
-      <c r="C25" s="8" t="n">
+      <c r="C25" s="7" t="n">
         <v>0.42</v>
       </c>
-      <c r="D25" s="8" t="n">
+      <c r="D25" s="7" t="n">
         <v>4.691</v>
       </c>
     </row>
@@ -2339,13 +2488,13 @@
           <t>San Francisco Giants</t>
         </is>
       </c>
-      <c r="B26" s="8" t="n">
+      <c r="B26" s="7" t="n">
         <v>0.305</v>
       </c>
-      <c r="C26" s="8" t="n">
+      <c r="C26" s="7" t="n">
         <v>0.396</v>
       </c>
-      <c r="D26" s="8" t="n">
+      <c r="D26" s="7" t="n">
         <v>4.278</v>
       </c>
     </row>
@@ -2355,13 +2504,13 @@
           <t>Seattle Mariners</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n">
+      <c r="B27" s="7" t="n">
         <v>0.311</v>
       </c>
-      <c r="C27" s="8" t="n">
+      <c r="C27" s="7" t="n">
         <v>0.376</v>
       </c>
-      <c r="D27" s="8" t="n">
+      <c r="D27" s="7" t="n">
         <v>4.173</v>
       </c>
     </row>
@@ -2371,13 +2520,13 @@
           <t>St. Louis Cardinals</t>
         </is>
       </c>
-      <c r="B28" s="8" t="n">
+      <c r="B28" s="7" t="n">
         <v>0.312</v>
       </c>
-      <c r="C28" s="8" t="n">
+      <c r="C28" s="7" t="n">
         <v>0.392</v>
       </c>
-      <c r="D28" s="8" t="n">
+      <c r="D28" s="7" t="n">
         <v>4.148</v>
       </c>
     </row>
@@ -2387,13 +2536,13 @@
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="B29" s="8" t="n">
+      <c r="B29" s="7" t="n">
         <v>0.302</v>
       </c>
-      <c r="C29" s="8" t="n">
+      <c r="C29" s="7" t="n">
         <v>0.366</v>
       </c>
-      <c r="D29" s="8" t="n">
+      <c r="D29" s="7" t="n">
         <v>3.728</v>
       </c>
     </row>
@@ -2403,13 +2552,13 @@
           <t>Texas Rangers</t>
         </is>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="7" t="n">
         <v>0.305</v>
       </c>
-      <c r="C30" s="8" t="n">
+      <c r="C30" s="7" t="n">
         <v>0.38</v>
       </c>
-      <c r="D30" s="8" t="n">
+      <c r="D30" s="7" t="n">
         <v>4.216</v>
       </c>
     </row>
@@ -2419,13 +2568,13 @@
           <t>Toronto Blue Jays</t>
         </is>
       </c>
-      <c r="B31" s="8" t="n">
+      <c r="B31" s="7" t="n">
         <v>0.313</v>
       </c>
-      <c r="C31" s="8" t="n">
+      <c r="C31" s="7" t="n">
         <v>0.389</v>
       </c>
-      <c r="D31" s="8" t="n">
+      <c r="D31" s="7" t="n">
         <v>4.142</v>
       </c>
     </row>
@@ -2435,92 +2584,97 @@
           <t>Washington Nationals</t>
         </is>
       </c>
-      <c r="B32" s="8" t="n">
+      <c r="B32" s="7" t="n">
         <v>0.309</v>
       </c>
-      <c r="C32" s="8" t="n">
+      <c r="C32" s="7" t="n">
         <v>0.375</v>
       </c>
-      <c r="D32" s="8" t="n">
+      <c r="D32" s="7" t="n">
         <v>4.074</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>Select a single cell and type each INDEX(LINEST(...)) formula; there is no need to fill a block or press anything other than Enter.</t>
+          <t>Select a single cell and type each formula; there is no need to fill a block or press anything other than Enter.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H3">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(ISNUMBER(G3),ABS(G3-(18.910622))&lt;=MAX(0.02*ABS(18.910622),0.02))</formula>
+      <formula>AND(ISNUMBER(G3),ABS(G3-(CORREL($B$3:$B$32,$C$3:$C$32)))&lt;=MAX(0.02*ABS(CORREL($B$3:$B$32,$C$3:$C$32)),0.005))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>AND(ISNUMBER(G4),ABS(G4-(9.290201))&lt;=MAX(0.02*ABS(9.290201),0.02))</formula>
+      <formula>AND(ISNUMBER(G4),ABS(G4-(SLOPE($D$3:$D$32,$B$3:$B$32)))&lt;=MAX(0.02*ABS(SLOPE($D$3:$D$32,$B$3:$B$32)),0.05))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>AND(ISNUMBER(G5),ABS(G5-(-5.210607))&lt;=MAX(0.02*ABS(-5.210607),0.02))</formula>
+      <formula>AND(ISNUMBER(G5),ABS(G5-(RSQ($D$3:$D$32,$B$3:$B$32)))&lt;=MAX(0.02*ABS(RSQ($D$3:$D$32,$B$3:$B$32)),0.005))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6">
     <cfRule type="expression" priority="4" dxfId="0">
-      <formula>AND(ISNUMBER(G6),ABS(G6-(3.816157))&lt;=MAX(0.02*ABS(3.816157),0.01))</formula>
+      <formula>AND(ISNUMBER(G6),ABS(G6-(SLOPE($D$3:$D$32,$C$3:$C$32)))&lt;=MAX(0.02*ABS(SLOPE($D$3:$D$32,$C$3:$C$32)),0.05))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
     <cfRule type="expression" priority="5" dxfId="0">
-      <formula>AND(ISNUMBER(G7),ABS(G7-(1.941532))&lt;=MAX(0.02*ABS(1.941532),0.01))</formula>
+      <formula>AND(ISNUMBER(G7),ABS(G7-(RSQ($D$3:$D$32,$C$3:$C$32)))&lt;=MAX(0.02*ABS(RSQ($D$3:$D$32,$C$3:$C$32)),0.005))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8">
     <cfRule type="expression" priority="6" dxfId="0">
-      <formula>AND(ISNUMBER(G8),ABS(G8-(4.95541))&lt;=MAX(0.02*ABS(4.95541),0.01))</formula>
+      <formula>AND(ISNUMBER(G8),ABS(G8-(18.910622))&lt;=MAX(0.02*ABS(18.910622),0.02))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
     <cfRule type="expression" priority="7" dxfId="0">
-      <formula>AND(ISNUMBER(G9),ABS(G9-(4.78498))&lt;=MAX(0.02*ABS(4.78498),0.01))</formula>
+      <formula>AND(ISNUMBER(G9),ABS(G9-(9.290201))&lt;=MAX(0.02*ABS(9.290201),0.02))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10">
     <cfRule type="expression" priority="8" dxfId="0">
-      <formula>AND(ISNUMBER(G10),ABS(G10-(0.0000343))&lt;=MAX(0.02*ABS(0.0000343),0.0005))</formula>
+      <formula>AND(ISNUMBER(G10),ABS(G10-(-5.210607))&lt;=MAX(0.02*ABS(-5.210607),0.02))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
     <cfRule type="expression" priority="9" dxfId="0">
-      <formula>AND(ISNUMBER(G11),ABS(G11-(0.0000543))&lt;=MAX(0.02*ABS(0.0000543),0.0005))</formula>
+      <formula>AND(ISNUMBER(G11),ABS(G11-(3.816157))&lt;=MAX(0.02*ABS(3.816157),0.01))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H12">
     <cfRule type="expression" priority="10" dxfId="0">
-      <formula>AND(ISNUMBER(G12),ABS(G12-(0.926295))&lt;=MAX(0.02*ABS(0.926295),0.005))</formula>
+      <formula>AND(ISNUMBER(G12),ABS(G12-(1.941532))&lt;=MAX(0.02*ABS(1.941532),0.01))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
     <cfRule type="expression" priority="11" dxfId="0">
-      <formula>AND(ISNUMBER(G13),ABS(G13-(_xlfn.STDEV.S($B$3:$B$32)))&lt;=MAX(0.02*ABS(_xlfn.STDEV.S($B$3:$B$32)),0.0002))</formula>
+      <formula>AND(ISNUMBER(G13),ABS(G13-(4.95541))&lt;=MAX(0.02*ABS(4.95541),0.01))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14">
     <cfRule type="expression" priority="12" dxfId="0">
-      <formula>AND(ISNUMBER(G14),ABS(G14-(_xlfn.STDEV.S($C$3:$C$32)))&lt;=MAX(0.02*ABS(_xlfn.STDEV.S($C$3:$C$32)),0.0002))</formula>
+      <formula>AND(ISNUMBER(G14),ABS(G14-(4.78498))&lt;=MAX(0.02*ABS(4.78498),0.01))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15">
     <cfRule type="expression" priority="13" dxfId="0">
-      <formula>AND(ISNUMBER(G15),ABS(G15-(0.236701))&lt;=MAX(0.02*ABS(0.236701),0.005))</formula>
+      <formula>AND(ISNUMBER(G15),ABS(G15-(0.0000343))&lt;=MAX(0.02*ABS(0.0000343),0.0005))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
     <cfRule type="expression" priority="14" dxfId="0">
-      <formula>AND(ISNUMBER(G16),ABS(G16-(0.228561))&lt;=MAX(0.02*ABS(0.228561),0.005))</formula>
+      <formula>AND(ISNUMBER(G16),ABS(G16-(0.0000543))&lt;=MAX(0.02*ABS(0.0000543),0.0005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="expression" priority="15" dxfId="0">
+      <formula>AND(ISNUMBER(G17),ABS(G17-(0.926295))&lt;=MAX(0.02*ABS(0.926295),0.005))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Week 5 sheet 2: plain-English labels and fewer formulas to type
</commit_message>
<xml_diff>
--- a/weeks/week05/data/hand-build-regression-worksheet.xlsx
+++ b/weeks/week05/data/hand-build-regression-worksheet.xlsx
@@ -68,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -78,6 +78,9 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -1202,14 +1205,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="3" customWidth="1" min="8" max="8"/>
@@ -1509,190 +1512,318 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Slope, SLOPE(y range, x range)</t>
+    <row r="15" ht="34" customHeight="1">
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Slope: points of margin that go with one more rush attempt.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=SLOPE(D3:D12, B3:B12)   margin, then rush attempts</t>
+          </r>
         </is>
       </c>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="5" t="n"/>
     </row>
-    <row r="16">
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Intercept, INTERCEPT(y range, x range)</t>
+    <row r="16" ht="34" customHeight="1">
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Intercept: the margin the line predicts at zero rush attempts.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=INTERCEPT(D3:D12, B3:B12)</t>
+          </r>
         </is>
       </c>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="5" t="n"/>
     </row>
-    <row r="17">
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Sum of squared residuals</t>
+    <row r="17" ht="34" customHeight="1">
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">How far off the line is in total: add up the squared misses.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=SUM(G3:G12)   the residual squared column</t>
+          </r>
         </is>
       </c>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="5" t="n"/>
     </row>
-    <row r="18">
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Residual standard error: SQRT of that sum divided by (n minus 2), n = 10</t>
+    <row r="18" ht="34" customHeight="1">
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">The typical miss, in points of margin (residual standard error).
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=SQRT(sum of squared misses / (n - 2))   n = 10 games</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="5" t="n"/>
     </row>
-    <row r="19">
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Check it with Excel, STEYX(y range, x range)</t>
+    <row r="19" ht="64" customHeight="1">
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Standard error of the slope: how much the slope would move if you drew ten different games. Bigger misses raise it; more spread in rush attempts lowers it.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=typical miss / SQRT(DEVSQ(B3:B12))</t>
+          </r>
         </is>
       </c>
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="5" t="n"/>
     </row>
-    <row r="20">
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Standard error of the slope: residual standard error divided by SQRT of the sum of squared x deviations</t>
+    <row r="20" ht="34" customHeight="1">
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">t: how many standard errors the slope sits away from zero.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=slope / standard error</t>
+          </r>
         </is>
       </c>
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="5" t="n"/>
     </row>
-    <row r="21">
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>t: slope divided by its standard error</t>
+    <row r="21" ht="49" customHeight="1">
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">p-value: if rushing had no link to margin, how often luck alone would give a slope at least this far from zero.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=T.DIST.2T(ABS(t), n - 2)</t>
+          </r>
         </is>
       </c>
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="5" t="n"/>
     </row>
-    <row r="22">
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>p-value, two-sided: T.DIST.2T(ABS(t), n minus 2)</t>
+    <row r="22" ht="49" customHeight="1">
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Low end of the 95% range: the smallest slope these ten games still allow.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=slope - T.INV.2T(0.05, n - 2) * standard error</t>
+          </r>
         </is>
       </c>
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="5" t="n"/>
     </row>
-    <row r="23">
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Lower end of the 95% interval: slope minus T.INV.2T(0.05, n minus 2) times the standard error</t>
+    <row r="23" ht="34" customHeight="1">
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">High end of the 95% range: the largest slope they still allow.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=slope + T.INV.2T(0.05, n - 2) * standard error</t>
+          </r>
         </is>
       </c>
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="5" t="n"/>
     </row>
-    <row r="24">
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Upper end of the 95% interval</t>
+    <row r="24" ht="49" customHeight="1">
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Now turnover differential instead: points of margin per extra turnover won.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=SLOPE(D3:D12, C3:C12)</t>
+          </r>
         </is>
       </c>
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="5" t="n"/>
     </row>
-    <row r="25">
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Standard error of the slope from Excel, INDEX(LINEST(y range, x range, TRUE, TRUE), 2, 1)</t>
+    <row r="25" ht="34" customHeight="1">
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Its standard error, in one step this time.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=INDEX(LINEST(D3:D12, C3:C12, TRUE, TRUE), 2, 1)</t>
+          </r>
         </is>
       </c>
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="5" t="n"/>
     </row>
-    <row r="26">
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Turnover differential as x instead: its slope, SLOPE(y range, turnover range)</t>
+    <row r="26" ht="34" customHeight="1">
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Its p-value.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=T.DIST.2T(ABS(slope / standard error), n - 2)</t>
+          </r>
         </is>
       </c>
       <c r="F26" s="6" t="n"/>
       <c r="G26" s="5" t="n"/>
     </row>
-    <row r="27">
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Its standard error, INDEX(LINEST(y range, turnover range, TRUE, TRUE), 2, 1)</t>
+    <row r="27" ht="34" customHeight="1">
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Points of margin that go with a typical swing in rush attempts.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=rush slope * STDEV.S(B3:B12)</t>
+          </r>
         </is>
       </c>
       <c r="F27" s="6" t="n"/>
       <c r="G27" s="5" t="n"/>
     </row>
-    <row r="28">
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Its p-value, two-sided: T.DIST.2T(ABS(slope divided by standard error), n minus 2)</t>
+    <row r="28" ht="49" customHeight="1">
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Points of margin that go with a typical swing in turnover differential.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <color rgb="0000539F"/>
+            </rPr>
+            <t>=turnover slope * STDEV.S(C3:C12)</t>
+          </r>
         </is>
       </c>
       <c r="F28" s="6" t="n"/>
       <c r="G28" s="5" t="n"/>
     </row>
-    <row r="29">
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Lower end of its 95% interval</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="5" t="n"/>
-    </row>
     <row r="30">
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Upper end of its 95% interval</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="5" t="n"/>
-    </row>
-    <row r="31">
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Standard deviation of rush attempts across the ten games, STDEV.S</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="5" t="n"/>
-    </row>
-    <row r="32">
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Standard deviation of turnover differential, STDEV.S</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="5" t="n"/>
-    </row>
-    <row r="33">
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Margin moved by one standard deviation of rush attempts: the rush slope times that standard deviation</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="5" t="n"/>
-    </row>
-    <row r="34">
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Margin moved by one standard deviation of turnover differential</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="5" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="inlineStr">
-        <is>
-          <t>Every number in the first block is one Excel prints when you run Data Analysis, Regression, or LINEST. Build each one yourself, then confirm the standard error against LINEST.</t>
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Build the rushing numbers by hand. The Check column turns green when a cell is right.</t>
         </is>
       </c>
     </row>
@@ -1869,82 +2000,52 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G19">
     <cfRule type="expression" priority="35" dxfId="0">
-      <formula>AND(ISNUMBER(F19),ABS(F19-(STEYX($D$3:$D$12,$B$3:$B$12)))&lt;=MAX(0.02*ABS(STEYX($D$3:$D$12,$B$3:$B$12)),0.05))</formula>
+      <formula>AND(ISNUMBER(F19),ABS(F19-((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))))&lt;=MAX(0.02*ABS((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))),0.005))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G20">
     <cfRule type="expression" priority="36" dxfId="0">
-      <formula>AND(ISNUMBER(F20),ABS(F20-((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))))&lt;=MAX(0.02*ABS((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))),0.005))</formula>
+      <formula>AND(ISNUMBER(F20),ABS(F20-((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G21">
     <cfRule type="expression" priority="37" dxfId="0">
-      <formula>AND(ISNUMBER(F21),ABS(F21-((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
+      <formula>AND(ISNUMBER(F21),ABS(F21-(_xlfn.T.DIST.2T(ABS((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),8)))&lt;=MAX(0.02*ABS(_xlfn.T.DIST.2T(ABS((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),8)),0.005))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G22">
     <cfRule type="expression" priority="38" dxfId="0">
-      <formula>AND(ISNUMBER(F22),ABS(F22-(_xlfn.T.DIST.2T(ABS((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),8)))&lt;=MAX(0.02*ABS(_xlfn.T.DIST.2T(ABS((SLOPE($D$3:$D$12,$B$3:$B$12)/(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),8)),0.005))</formula>
+      <formula>AND(ISNUMBER(F22),ABS(F22-((SLOPE($D$3:$D$12,$B$3:$B$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G23">
     <cfRule type="expression" priority="39" dxfId="0">
-      <formula>AND(ISNUMBER(F23),ABS(F23-((SLOPE($D$3:$D$12,$B$3:$B$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
+      <formula>AND(ISNUMBER(F23),ABS(F23-((SLOPE($D$3:$D$12,$B$3:$B$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G24">
     <cfRule type="expression" priority="40" dxfId="0">
-      <formula>AND(ISNUMBER(F24),ABS(F24-((SLOPE($D$3:$D$12,$B$3:$B$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12))))),0.01))</formula>
+      <formula>AND(ISNUMBER(F24),ABS(F24-(SLOPE($D$3:$D$12,$C$3:$C$12)))&lt;=MAX(0.02*ABS(SLOPE($D$3:$D$12,$C$3:$C$12)),0.01))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G25">
     <cfRule type="expression" priority="41" dxfId="0">
-      <formula>AND(ISNUMBER(F25),ABS(F25-((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))))&lt;=MAX(0.02*ABS((STEYX($D$3:$D$12,$B$3:$B$12)/SQRT(DEVSQ($B$3:$B$12)))),0.005))</formula>
+      <formula>AND(ISNUMBER(F25),ABS(F25-((STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))))&lt;=MAX(0.02*ABS((STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))),0.01))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G26">
     <cfRule type="expression" priority="42" dxfId="0">
-      <formula>AND(ISNUMBER(F26),ABS(F26-(SLOPE($D$3:$D$12,$C$3:$C$12)))&lt;=MAX(0.02*ABS(SLOPE($D$3:$D$12,$C$3:$C$12)),0.01))</formula>
+      <formula>AND(ISNUMBER(F26),ABS(F26-(_xlfn.T.DIST.2T(ABS(SLOPE($D$3:$D$12,$C$3:$C$12)/(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))),8)))&lt;=MAX(0.02*ABS(_xlfn.T.DIST.2T(ABS(SLOPE($D$3:$D$12,$C$3:$C$12)/(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))),8)),0.005))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G27">
     <cfRule type="expression" priority="43" dxfId="0">
-      <formula>AND(ISNUMBER(F27),ABS(F27-((STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))))&lt;=MAX(0.02*ABS((STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))),0.01))</formula>
+      <formula>AND(ISNUMBER(F27),ABS(F27-((SLOPE($D$3:$D$12,$B$3:$B$12)*_xlfn.STDEV.S($B$3:$B$12))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)*_xlfn.STDEV.S($B$3:$B$12))),0.05))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G28">
     <cfRule type="expression" priority="44" dxfId="0">
-      <formula>AND(ISNUMBER(F28),ABS(F28-(_xlfn.T.DIST.2T(ABS(SLOPE($D$3:$D$12,$C$3:$C$12)/(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))),8)))&lt;=MAX(0.02*ABS(_xlfn.T.DIST.2T(ABS(SLOPE($D$3:$D$12,$C$3:$C$12)/(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12)))),8)),0.005))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G29">
-    <cfRule type="expression" priority="45" dxfId="0">
-      <formula>AND(ISNUMBER(F29),ABS(F29-((SLOPE($D$3:$D$12,$C$3:$C$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$C$3:$C$12)-_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12))))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G30">
-    <cfRule type="expression" priority="46" dxfId="0">
-      <formula>AND(ISNUMBER(F30),ABS(F30-((SLOPE($D$3:$D$12,$C$3:$C$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12))))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$C$3:$C$12)+_xlfn.T.INV.2T(0.05,8)*(STEYX($D$3:$D$12,$C$3:$C$12)/SQRT(DEVSQ($C$3:$C$12))))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G31">
-    <cfRule type="expression" priority="47" dxfId="0">
-      <formula>AND(ISNUMBER(F31),ABS(F31-(_xlfn.STDEV.S($B$3:$B$12)))&lt;=MAX(0.02*ABS(_xlfn.STDEV.S($B$3:$B$12)),0.01))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G32">
-    <cfRule type="expression" priority="48" dxfId="0">
-      <formula>AND(ISNUMBER(F32),ABS(F32-(_xlfn.STDEV.S($C$3:$C$12)))&lt;=MAX(0.02*ABS(_xlfn.STDEV.S($C$3:$C$12)),0.01))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G33">
-    <cfRule type="expression" priority="49" dxfId="0">
-      <formula>AND(ISNUMBER(F33),ABS(F33-((SLOPE($D$3:$D$12,$B$3:$B$12)*_xlfn.STDEV.S($B$3:$B$12))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$B$3:$B$12)*_xlfn.STDEV.S($B$3:$B$12))),0.05))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G34">
-    <cfRule type="expression" priority="50" dxfId="0">
-      <formula>AND(ISNUMBER(F34),ABS(F34-((SLOPE($D$3:$D$12,$C$3:$C$12)*_xlfn.STDEV.S($C$3:$C$12))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$C$3:$C$12)*_xlfn.STDEV.S($C$3:$C$12))),0.05))</formula>
+      <formula>AND(ISNUMBER(F28),ABS(F28-((SLOPE($D$3:$D$12,$C$3:$C$12)*_xlfn.STDEV.S($C$3:$C$12))))&lt;=MAX(0.02*ABS((SLOPE($D$3:$D$12,$C$3:$C$12)*_xlfn.STDEV.S($C$3:$C$12))),0.05))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2015,13 +2116,13 @@
           <t>Arizona Diamondbacks</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
+      <c r="B3" s="8" t="n">
         <v>0.337</v>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C3" s="8" t="n">
         <v>0.44</v>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="8" t="n">
         <v>5.469</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -2029,7 +2130,7 @@
           <t>How closely OBP and SLG move together across the 30 teams, CORREL(OBP range, SLG range)</t>
         </is>
       </c>
-      <c r="G3" s="8" t="n"/>
+      <c r="G3" s="9" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -2038,13 +2139,13 @@
           <t>Atlanta Braves</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="8" t="n">
         <v>0.309</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="8" t="n">
         <v>0.415</v>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="8" t="n">
         <v>4.346</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -2052,7 +2153,7 @@
           <t>OBP alone: its slope, SLOPE(y range, OBP range)</t>
         </is>
       </c>
-      <c r="G4" s="8" t="n"/>
+      <c r="G4" s="9" t="n"/>
       <c r="H4" s="5" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
@@ -2061,13 +2162,13 @@
           <t>Baltimore Orioles</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>0.315</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="8" t="n">
         <v>0.435</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="8" t="n">
         <v>4.852</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2075,7 +2176,7 @@
           <t>OBP alone: R squared, RSQ(y range, OBP range)</t>
         </is>
       </c>
-      <c r="G5" s="8" t="n"/>
+      <c r="G5" s="9" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
     <row r="6" ht="32" customHeight="1">
@@ -2084,13 +2185,13 @@
           <t>Boston Red Sox</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>0.319</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <v>0.423</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="8" t="n">
         <v>4.636</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2098,7 +2199,7 @@
           <t>SLG alone: its slope, SLOPE(y range, SLG range)</t>
         </is>
       </c>
-      <c r="G6" s="8" t="n"/>
+      <c r="G6" s="9" t="n"/>
       <c r="H6" s="5" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -2107,13 +2208,13 @@
           <t>Chicago Cubs</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>0.317</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="8" t="n">
         <v>0.393</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <v>4.543</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2121,7 +2222,7 @@
           <t>SLG alone: R squared, RSQ(y range, SLG range)</t>
         </is>
       </c>
-      <c r="G7" s="8" t="n"/>
+      <c r="G7" s="9" t="n"/>
       <c r="H7" s="5" t="n"/>
     </row>
     <row r="8" ht="32" customHeight="1">
@@ -2130,13 +2231,13 @@
           <t>Chicago White Sox</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>0.278</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
         <v>0.34</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <v>3.13</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2144,7 +2245,7 @@
           <t>Both together. Coefficient on OBP: INDEX(LINEST(y range, both x columns, TRUE, TRUE), 1, 2). LINEST lists the x coefficients in reverse column order.</t>
         </is>
       </c>
-      <c r="G8" s="8" t="n"/>
+      <c r="G8" s="9" t="n"/>
       <c r="H8" s="5" t="n"/>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -2153,13 +2254,13 @@
           <t>Cincinnati Reds</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>0.305</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="8" t="n">
         <v>0.388</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="8" t="n">
         <v>4.315</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -2167,7 +2268,7 @@
           <t>Coefficient on SLG: INDEX(LINEST(...), 1, 1)</t>
         </is>
       </c>
-      <c r="G9" s="8" t="n"/>
+      <c r="G9" s="9" t="n"/>
       <c r="H9" s="5" t="n"/>
     </row>
     <row r="10" ht="32" customHeight="1">
@@ -2176,13 +2277,13 @@
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="8" t="n">
         <v>0.307</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="8" t="n">
         <v>0.395</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="8" t="n">
         <v>4.398</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2190,7 +2291,7 @@
           <t>Intercept: INDEX(LINEST(...), 1, 3)</t>
         </is>
       </c>
-      <c r="G10" s="8" t="n"/>
+      <c r="G10" s="9" t="n"/>
       <c r="H10" s="5" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
@@ -2199,13 +2300,13 @@
           <t>Colorado Rockies</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <v>0.304</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="8" t="n">
         <v>0.4</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="8" t="n">
         <v>4.21</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2213,7 +2314,7 @@
           <t>Standard error of the OBP coefficient: INDEX(LINEST(...), 2, 2)</t>
         </is>
       </c>
-      <c r="G11" s="8" t="n"/>
+      <c r="G11" s="9" t="n"/>
       <c r="H11" s="5" t="n"/>
     </row>
     <row r="12" ht="32" customHeight="1">
@@ -2222,13 +2323,13 @@
           <t>Detroit Tigers</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="8" t="n">
         <v>0.3</v>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="8" t="n">
         <v>0.385</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="8" t="n">
         <v>4.21</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2236,7 +2337,7 @@
           <t>Standard error of the SLG coefficient: INDEX(LINEST(...), 2, 1)</t>
         </is>
       </c>
-      <c r="G12" s="8" t="n"/>
+      <c r="G12" s="9" t="n"/>
       <c r="H12" s="5" t="n"/>
     </row>
     <row r="13" ht="32" customHeight="1">
@@ -2245,13 +2346,13 @@
           <t>Houston Astros</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="8" t="n">
         <v>0.322</v>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="8" t="n">
         <v>0.418</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="8" t="n">
         <v>4.596</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -2259,7 +2360,7 @@
           <t>t for OBP: coefficient divided by its standard error</t>
         </is>
       </c>
-      <c r="G13" s="8" t="n"/>
+      <c r="G13" s="9" t="n"/>
       <c r="H13" s="5" t="n"/>
     </row>
     <row r="14" ht="32" customHeight="1">
@@ -2268,13 +2369,13 @@
           <t>Kansas City Royals</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="8" t="n">
         <v>0.306</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="8" t="n">
         <v>0.403</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="8" t="n">
         <v>4.537</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -2282,7 +2383,7 @@
           <t>t for SLG</t>
         </is>
       </c>
-      <c r="G14" s="8" t="n"/>
+      <c r="G14" s="9" t="n"/>
       <c r="H14" s="5" t="n"/>
     </row>
     <row r="15" ht="32" customHeight="1">
@@ -2291,13 +2392,13 @@
           <t>Los Angeles Angels</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="8" t="n">
         <v>0.301</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="8" t="n">
         <v>0.369</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="8" t="n">
         <v>3.92</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -2305,7 +2406,7 @@
           <t>p-value for OBP: T.DIST.2T(ABS(t), n minus 3), n = 30</t>
         </is>
       </c>
-      <c r="G15" s="8" t="n"/>
+      <c r="G15" s="9" t="n"/>
       <c r="H15" s="5" t="n"/>
     </row>
     <row r="16" ht="32" customHeight="1">
@@ -2314,13 +2415,13 @@
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="8" t="n">
         <v>0.335</v>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="8" t="n">
         <v>0.446</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="8" t="n">
         <v>5.198</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -2328,7 +2429,7 @@
           <t>p-value for SLG</t>
         </is>
       </c>
-      <c r="G16" s="8" t="n"/>
+      <c r="G16" s="9" t="n"/>
       <c r="H16" s="5" t="n"/>
     </row>
     <row r="17" ht="32" customHeight="1">
@@ -2337,13 +2438,13 @@
           <t>Miami Marlins</t>
         </is>
       </c>
-      <c r="B17" s="7" t="n">
+      <c r="B17" s="8" t="n">
         <v>0.3</v>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="8" t="n">
         <v>0.378</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="8" t="n">
         <v>3.932</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -2351,7 +2452,7 @@
           <t>R squared with both: INDEX(LINEST(...), 3, 1)</t>
         </is>
       </c>
-      <c r="G17" s="8" t="n"/>
+      <c r="G17" s="9" t="n"/>
       <c r="H17" s="5" t="n"/>
     </row>
     <row r="18">
@@ -2360,13 +2461,13 @@
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="8" t="n">
         <v>0.326</v>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="8" t="n">
         <v>0.403</v>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="8" t="n">
         <v>4.796</v>
       </c>
     </row>
@@ -2376,13 +2477,13 @@
           <t>Minnesota Twins</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B19" s="8" t="n">
         <v>0.315</v>
       </c>
-      <c r="C19" s="7" t="n">
+      <c r="C19" s="8" t="n">
         <v>0.411</v>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="8" t="n">
         <v>4.58</v>
       </c>
     </row>
@@ -2392,13 +2493,13 @@
           <t>New York Mets</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n">
+      <c r="B20" s="8" t="n">
         <v>0.319</v>
       </c>
-      <c r="C20" s="7" t="n">
+      <c r="C20" s="8" t="n">
         <v>0.415</v>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="8" t="n">
         <v>4.741</v>
       </c>
     </row>
@@ -2408,13 +2509,13 @@
           <t>New York Yankees</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="8" t="n">
         <v>0.333</v>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="C21" s="8" t="n">
         <v>0.429</v>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="8" t="n">
         <v>5.031</v>
       </c>
     </row>
@@ -2424,13 +2525,13 @@
           <t>Oakland Athletics</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B22" s="8" t="n">
         <v>0.301</v>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="8" t="n">
         <v>0.393</v>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="8" t="n">
         <v>3.969</v>
       </c>
     </row>
@@ -2440,13 +2541,13 @@
           <t>Philadelphia Phillies</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B23" s="8" t="n">
         <v>0.325</v>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="8" t="n">
         <v>0.425</v>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="8" t="n">
         <v>4.84</v>
       </c>
     </row>
@@ -2456,13 +2557,13 @@
           <t>Pittsburgh Pirates</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n">
+      <c r="B24" s="8" t="n">
         <v>0.301</v>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="8" t="n">
         <v>0.371</v>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="8" t="n">
         <v>4.105</v>
       </c>
     </row>
@@ -2472,13 +2573,13 @@
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n">
+      <c r="B25" s="8" t="n">
         <v>0.324</v>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C25" s="8" t="n">
         <v>0.42</v>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="D25" s="8" t="n">
         <v>4.691</v>
       </c>
     </row>
@@ -2488,13 +2589,13 @@
           <t>San Francisco Giants</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n">
+      <c r="B26" s="8" t="n">
         <v>0.305</v>
       </c>
-      <c r="C26" s="7" t="n">
+      <c r="C26" s="8" t="n">
         <v>0.396</v>
       </c>
-      <c r="D26" s="7" t="n">
+      <c r="D26" s="8" t="n">
         <v>4.278</v>
       </c>
     </row>
@@ -2504,13 +2605,13 @@
           <t>Seattle Mariners</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n">
+      <c r="B27" s="8" t="n">
         <v>0.311</v>
       </c>
-      <c r="C27" s="7" t="n">
+      <c r="C27" s="8" t="n">
         <v>0.376</v>
       </c>
-      <c r="D27" s="7" t="n">
+      <c r="D27" s="8" t="n">
         <v>4.173</v>
       </c>
     </row>
@@ -2520,13 +2621,13 @@
           <t>St. Louis Cardinals</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n">
+      <c r="B28" s="8" t="n">
         <v>0.312</v>
       </c>
-      <c r="C28" s="7" t="n">
+      <c r="C28" s="8" t="n">
         <v>0.392</v>
       </c>
-      <c r="D28" s="7" t="n">
+      <c r="D28" s="8" t="n">
         <v>4.148</v>
       </c>
     </row>
@@ -2536,13 +2637,13 @@
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n">
+      <c r="B29" s="8" t="n">
         <v>0.302</v>
       </c>
-      <c r="C29" s="7" t="n">
+      <c r="C29" s="8" t="n">
         <v>0.366</v>
       </c>
-      <c r="D29" s="7" t="n">
+      <c r="D29" s="8" t="n">
         <v>3.728</v>
       </c>
     </row>
@@ -2552,13 +2653,13 @@
           <t>Texas Rangers</t>
         </is>
       </c>
-      <c r="B30" s="7" t="n">
+      <c r="B30" s="8" t="n">
         <v>0.305</v>
       </c>
-      <c r="C30" s="7" t="n">
+      <c r="C30" s="8" t="n">
         <v>0.38</v>
       </c>
-      <c r="D30" s="7" t="n">
+      <c r="D30" s="8" t="n">
         <v>4.216</v>
       </c>
     </row>
@@ -2568,13 +2669,13 @@
           <t>Toronto Blue Jays</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n">
+      <c r="B31" s="8" t="n">
         <v>0.313</v>
       </c>
-      <c r="C31" s="7" t="n">
+      <c r="C31" s="8" t="n">
         <v>0.389</v>
       </c>
-      <c r="D31" s="7" t="n">
+      <c r="D31" s="8" t="n">
         <v>4.142</v>
       </c>
     </row>
@@ -2584,13 +2685,13 @@
           <t>Washington Nationals</t>
         </is>
       </c>
-      <c r="B32" s="7" t="n">
+      <c r="B32" s="8" t="n">
         <v>0.309</v>
       </c>
-      <c r="C32" s="7" t="n">
+      <c r="C32" s="8" t="n">
         <v>0.375</v>
       </c>
-      <c r="D32" s="7" t="n">
+      <c r="D32" s="8" t="n">
         <v>4.074</v>
       </c>
     </row>

</xml_diff>